<commit_message>
role changed to designations
</commit_message>
<xml_diff>
--- a/public/staff_allocation_template.xlsx
+++ b/public/staff_allocation_template.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Staff" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Projects" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Assignments" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Roles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Designations" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1949,68 +1949,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Role Code</t>
+          <t>Designation Code</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Role Name</t>
+          <t>Designation Name</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>RA</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Project Lead</t>
+          <t>Research Associate</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>SRA</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Member</t>
+          <t>Senior Research Associate</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>DOR</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Assisting</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>DOR</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Director of Research</t>
         </is>

</xml_diff>